<commit_message>
Se completa menu, ventas , inventario, productos
</commit_message>
<xml_diff>
--- a/documentos/BaseDatos.xlsx
+++ b/documentos/BaseDatos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mis-proyectos\gestion-minimarket\documentos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\personal\gestion-minimarket\documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FDBB7D6-3519-4979-87FB-D699917B4A10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49896FEE-68C2-42FA-9BA4-50B7BE555845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="4" xr2:uid="{90DC8E08-B72D-4FE1-934B-5D8DD9EE30BB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="5" xr2:uid="{90DC8E08-B72D-4FE1-934B-5D8DD9EE30BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -78,7 +78,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Jenrry Pena Cacya:</t>
         </r>
@@ -87,7 +87,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 unique constraint.</t>
@@ -102,7 +102,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Jenrry Pena Cacya:</t>
         </r>
@@ -111,7 +111,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 id product y medida venta es unique.</t>
@@ -184,7 +184,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Jenrry Pena Cacya:</t>
         </r>
@@ -193,7 +193,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 tiene que ser unico para la busqueda por codigo y codigo de barras.</t>
@@ -828,7 +828,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -848,14 +848,14 @@
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -864,19 +864,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
     <font>
       <i/>
@@ -1025,12 +1012,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>

</xml_diff>